<commit_message>
Deployed 598b8380 with MkDocs version: 1.6.0
</commit_message>
<xml_diff>
--- a/Manual/source/tab/parameters.xlsx
+++ b/Manual/source/tab/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="19"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="21"/>
   </bookViews>
   <sheets>
     <sheet name="TGZ-D-48-13_26" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,16 +28,18 @@
     <sheet name="TGZ-S-400-10_20" sheetId="18" state="visible" r:id="rId20"/>
     <sheet name="TGZ-S-400-14_30" sheetId="19" state="visible" r:id="rId21"/>
     <sheet name="TGZ-D-560-3_9" sheetId="20" state="visible" r:id="rId22"/>
-    <sheet name="TGZ-D-560-30_50" sheetId="21" state="visible" r:id="rId23"/>
-    <sheet name="TGS-320-10_15" sheetId="22" state="visible" r:id="rId24"/>
-    <sheet name="TGS-560-25_50" sheetId="23" state="visible" r:id="rId25"/>
-    <sheet name="TGS-560-50_100" sheetId="24" state="visible" r:id="rId26"/>
-    <sheet name="TGMmini" sheetId="25" state="visible" r:id="rId27"/>
-    <sheet name="TGMcontroller" sheetId="26" state="visible" r:id="rId28"/>
-    <sheet name="TGZpMotion" sheetId="27" state="visible" r:id="rId29"/>
-    <sheet name="commonHW_DI" sheetId="28" state="visible" r:id="rId30"/>
-    <sheet name="commonHW_DO" sheetId="29" state="visible" r:id="rId31"/>
-    <sheet name="commonHW_AI" sheetId="30" state="visible" r:id="rId32"/>
+    <sheet name="TGZ-D-560-7_15" sheetId="21" state="visible" r:id="rId23"/>
+    <sheet name="TGZ-D-560-10_20" sheetId="22" state="visible" r:id="rId24"/>
+    <sheet name="TGZ-D-560-30_50" sheetId="23" state="visible" r:id="rId25"/>
+    <sheet name="TGS-320-10_15" sheetId="24" state="visible" r:id="rId26"/>
+    <sheet name="TGS-560-25_50" sheetId="25" state="visible" r:id="rId27"/>
+    <sheet name="TGS-560-50_100" sheetId="26" state="visible" r:id="rId28"/>
+    <sheet name="TGMmini" sheetId="27" state="visible" r:id="rId29"/>
+    <sheet name="TGMcontroller" sheetId="28" state="visible" r:id="rId30"/>
+    <sheet name="TGZpMotion" sheetId="29" state="visible" r:id="rId31"/>
+    <sheet name="commonHW_DI" sheetId="30" state="visible" r:id="rId32"/>
+    <sheet name="commonHW_DO" sheetId="31" state="visible" r:id="rId33"/>
+    <sheet name="commonHW_AI" sheetId="32" state="visible" r:id="rId34"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -49,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="291">
   <si>
     <t xml:space="preserve">NAPÁJENÍ</t>
   </si>
@@ -4216,7 +4218,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4416,12 +4418,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4433,174 +4434,208 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C2" s="3"/>
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="C3" s="3"/>
+      <c r="A3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C4" s="3"/>
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C5" s="3"/>
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C6" s="3"/>
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C7" s="3"/>
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C8" s="3"/>
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C10" s="3"/>
+      <c r="A9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="C11" s="3"/>
+      <c r="A11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="3"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>186</v>
+        <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>188</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>189</v>
+        <v>158</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>1</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>190</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>191</v>
+        <v>31</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>128</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>193</v>
+        <v>33</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>194</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>195</v>
+        <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>196</v>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -4619,12 +4654,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4636,163 +4670,144 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>166</v>
+      <c r="A2" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="C2" s="3"/>
+        <v>153</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>168</v>
+      <c r="A3" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="3"/>
+        <v>154</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>170</v>
+      <c r="A4" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="C4" s="3"/>
+        <v>165</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>172</v>
+      <c r="A5" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C5" s="3"/>
+        <v>150</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>174</v>
+      <c r="A6" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="3"/>
+        <v>156</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>176</v>
+      <c r="A7" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C7" s="3"/>
+        <v>47</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>178</v>
+      <c r="A8" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="C8" s="3"/>
+        <v>157</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>180</v>
+      <c r="A9" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="C10" s="3"/>
+        <v>17</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>184</v>
+      <c r="A11" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="C11" s="3"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="3"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>186</v>
+        <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>188</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>189</v>
+        <v>158</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>1</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>190</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>191</v>
+        <v>31</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>204</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>192</v>
+        <v>33</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>1</v>
@@ -4800,18 +4815,63 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>193</v>
+        <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>1</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>195</v>
+        <v>36</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>196</v>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -4830,7 +4890,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
@@ -4847,206 +4907,174 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>153</v>
-      </c>
+      <c r="A2" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>205</v>
+        <v>168</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>169</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>46</v>
+        <v>170</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>171</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>198</v>
+        <v>172</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>173</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>174</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>175</v>
       </c>
       <c r="C6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>56</v>
+        <v>176</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>177</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>165</v>
+        <v>178</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>179</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>201</v>
+        <v>180</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>181</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>1</v>
+        <v>182</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>183</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>206</v>
+        <v>184</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>184</v>
+      <c r="A12" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>207</v>
+        <v>17</v>
       </c>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="3"/>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>188</v>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" s="1" t="s">
         <v>190</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>1</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>36</v>
+        <v>193</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B26" s="1" t="s">
         <v>196</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -5065,7 +5093,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
@@ -5082,65 +5110,71 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>212</v>
+      <c r="A2" s="3" t="s">
+        <v>166</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>214</v>
+      <c r="A3" s="3" t="s">
+        <v>168</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>1</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>216</v>
+      <c r="A4" s="3" t="s">
+        <v>170</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>199</v>
+      </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>18</v>
+      <c r="A6" s="3" t="s">
+        <v>174</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="C6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>217</v>
+      <c r="A7" s="3" t="s">
+        <v>176</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>218</v>
+        <v>200</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>219</v>
+      <c r="A8" s="3" t="s">
+        <v>178</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>220</v>
+        <v>201</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>19</v>
+      <c r="A9" s="3" t="s">
+        <v>180</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>1</v>
@@ -5148,83 +5182,110 @@
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>221</v>
+      <c r="A10" s="3" t="s">
+        <v>182</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>223</v>
+      <c r="A11" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>225</v>
+        <v>16</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>226</v>
+        <v>17</v>
       </c>
       <c r="C12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>186</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>227</v>
+        <v>187</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>1</v>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>229</v>
+        <v>28</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>230</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>19</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>233</v>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -5243,7 +5304,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
@@ -5261,150 +5322,205 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C2" s="3"/>
+        <v>153</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>214</v>
+      <c r="A3" s="3" t="s">
+        <v>166</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>216</v>
+      <c r="A4" s="3" t="s">
+        <v>168</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>46</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>198</v>
+      </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>18</v>
+      <c r="A6" s="3" t="s">
+        <v>172</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="C6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>21</v>
+      <c r="A7" s="3" t="s">
+        <v>174</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>23</v>
+      <c r="A8" s="3" t="s">
+        <v>176</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>165</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>19</v>
+      <c r="A9" s="3" t="s">
+        <v>178</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1</v>
+        <v>201</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>223</v>
+      <c r="A10" s="3" t="s">
+        <v>180</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>1</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>206</v>
+      </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>28</v>
+      <c r="A12" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1</v>
+        <v>207</v>
       </c>
       <c r="C12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>227</v>
+        <v>16</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>234</v>
+        <v>17</v>
       </c>
       <c r="C13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>229</v>
+        <v>187</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>37</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>189</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>99</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>103</v>
+      <c r="A19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>104</v>
+      <c r="A20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -5423,7 +5539,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
@@ -5480,19 +5596,19 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>217</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>22</v>
+        <v>218</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>219</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>220</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -5507,60 +5623,82 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="C13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="1" t="s">
+        <v>1</v>
+      </c>
       <c r="C14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1</v>
+        <v>228</v>
       </c>
       <c r="C15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>231</v>
-      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>191</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -5579,403 +5717,168 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="26.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="31.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="30.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>245</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>212</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>256</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>214</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>263</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
-        <v>1</v>
+      <c r="A4" s="1" t="s">
+        <v>216</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D4" s="1" t="n">
+        <v>213</v>
+      </c>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F5" s="1" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H5" s="1" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F6" s="1" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F7" s="1" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="G7" s="1" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H7" s="1" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="J7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" s="1" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F8" s="1" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="J8" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1" t="n">
-        <v>50</v>
-      </c>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
-        <v>6</v>
+      <c r="A9" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="F9" s="1" t="n">
-        <v>2.05</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H9" s="1" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="I9" s="1" t="n">
-        <v>8.2</v>
-      </c>
-      <c r="J9" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="1" t="n">
-        <v>50</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="n">
-        <v>7</v>
+      <c r="A10" s="1" t="s">
+        <v>223</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="F10" s="1" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G10" s="1" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="H10" s="1" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I10" s="1" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="J10" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1" t="n">
-        <v>50</v>
-      </c>
+        <v>224</v>
+      </c>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D11" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="F11" s="1" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G11" s="1" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="H11" s="1" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="I11" s="1" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="J11" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="K11" s="1" t="n">
-        <v>50</v>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -5994,278 +5897,144 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="26.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="31.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>276</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>212</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>282</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>214</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>263</v>
-      </c>
+        <v>215</v>
+      </c>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="1" t="n">
+      <c r="A4" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D4" s="1" t="n">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="H4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="E5" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="H5" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" s="1" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="E6" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="H6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="1" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="E7" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G7" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="H7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="I7" s="1" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="E8" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G8" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" s="1" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="E9" s="1" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G9" s="1" t="n">
-        <v>300</v>
-      </c>
-      <c r="H9" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" s="1" t="n">
-        <v>10</v>
+      <c r="B12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -6499,6 +6268,711 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="26.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="31.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="30.24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="J4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>8.2</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="F10" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I10" s="1" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="F11" s="1" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I11" s="1" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="1" t="n">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="26.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="31.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30.24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>24</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>28</v>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>300</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>

</xml_diff>

<commit_message>
Deployed 0f72989f with MkDocs version: 1.6.0
</commit_message>
<xml_diff>
--- a/Manual/source/tab/parameters.xlsx
+++ b/Manual/source/tab/parameters.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="301">
   <si>
     <t xml:space="preserve">NAPÁJENÍ</t>
   </si>
@@ -515,10 +515,64 @@
     <t xml:space="preserve">24 VDC ± 10 %, 2 A*</t>
   </si>
   <si>
+    <t xml:space="preserve">140-600 VDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,4 kW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 x 9 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VSTUPY/VÝSTUPY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 3pin WEIDMÜLLER BLZ 7.62HP/03/180LR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 5pin WEIDMÜLLER BCZ 3.81/05/180F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 x 6pin WEIDMÜLLER  BLZ 7.62HP/06/180LR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 x 8pin WEIDMÜLLER B2CF 3.50/08/180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 12pin WEIDMÜLLER B2CF 3.50/12/180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtr obsahující napájecí modul TGS-560-25/50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,8 kW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100 W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 kW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 x 20 A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150 W</t>
+  </si>
+  <si>
     <t xml:space="preserve">24-560 VDC</t>
   </si>
   <si>
-    <t xml:space="preserve">10kW</t>
+    <t xml:space="preserve">33 kW</t>
   </si>
   <si>
     <t xml:space="preserve">60 A</t>
@@ -527,9 +581,6 @@
     <t xml:space="preserve">900 W</t>
   </si>
   <si>
-    <t xml:space="preserve">VSTUPY/VÝSTUPY</t>
-  </si>
-  <si>
     <t xml:space="preserve">šroubovací svorky M8x12</t>
   </si>
   <si>
@@ -539,18 +590,9 @@
     <t xml:space="preserve">2 x 4pin  WEIDMÜLLER LSF</t>
   </si>
   <si>
-    <t xml:space="preserve">2 x 8pin WEIDMÜLLER B2CF 3.50/08/180</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 x 12pin WEIDMÜLLER B2CF 3.50/12/180</t>
-  </si>
-  <si>
     <t xml:space="preserve">Filtr obsahující napájecí modul TGS-560</t>
   </si>
   <si>
-    <t xml:space="preserve">33 kW</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vstupní napětí (VAC - 50/60 Hz) </t>
   </si>
   <si>
@@ -560,9 +602,6 @@
     <t xml:space="preserve">Maximální vstupní proud (AC) </t>
   </si>
   <si>
-    <t xml:space="preserve">16 A</t>
-  </si>
-  <si>
     <t xml:space="preserve">Výstupní napětí (DC) </t>
   </si>
   <si>
@@ -659,19 +698,10 @@
     <t xml:space="preserve">400 W</t>
   </si>
   <si>
-    <t xml:space="preserve">100 W</t>
-  </si>
-  <si>
     <t xml:space="preserve">32 A</t>
   </si>
   <si>
-    <t xml:space="preserve">1 x 5pin WEIDMÜLLER BCZ 3.81/05/180F</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 x 400 VAC/50Hz 63A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">150 W</t>
   </si>
   <si>
     <t xml:space="preserve">63 A</t>
@@ -3946,224 +3976,216 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="0" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="0" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>150</v>
+      <c r="B5" s="0" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="0" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>47</v>
+      <c r="B7" s="0" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>157</v>
+      <c r="B8" s="0" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="0" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="0" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="0" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="0" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="0" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="0" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="0" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>159</v>
+      <c r="B24" s="0" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>160</v>
+      <c r="B25" s="0" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>51</v>
+      <c r="B26" s="0" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>161</v>
+      <c r="A27" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
+      <c r="A28" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>163</v>
+      <c r="B28" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
+      <c r="A31" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>164</v>
+      <c r="B31" s="0" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4182,224 +4204,216 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="0" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>155</v>
+      <c r="B4" s="0" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>150</v>
+      <c r="B5" s="0" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>156</v>
+      <c r="B6" s="0" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>47</v>
+      <c r="B7" s="0" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>157</v>
+      <c r="B8" s="0" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="0" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="0" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="0" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="0" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="0" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="0" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="0" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>159</v>
+      <c r="B24" s="0" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>160</v>
+      <c r="B25" s="0" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>51</v>
+      <c r="B26" s="0" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>161</v>
+      <c r="A27" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
+      <c r="A28" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>163</v>
+      <c r="B28" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
+      <c r="A31" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>164</v>
+      <c r="B31" s="0" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4418,224 +4432,216 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="0" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="0" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>155</v>
+      <c r="B4" s="0" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>150</v>
+      <c r="B5" s="0" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>156</v>
+      <c r="B6" s="0" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>47</v>
+      <c r="B7" s="0" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>157</v>
+      <c r="B8" s="0" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="0" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="0" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="0" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="0" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="0" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="0" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="0" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="0" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="0" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="0" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>159</v>
+      <c r="B24" s="0" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>160</v>
+      <c r="B25" s="0" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>51</v>
+      <c r="B26" s="0" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>161</v>
+      <c r="A27" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
+      <c r="A28" s="0" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>163</v>
+      <c r="B28" s="0" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
+      <c r="A31" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>164</v>
+      <c r="B31" s="0" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -4682,7 +4688,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4690,7 +4696,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4706,7 +4712,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4722,7 +4728,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4767,7 +4773,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>1</v>
@@ -4818,7 +4824,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4826,7 +4832,7 @@
         <v>36</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4842,7 +4848,7 @@
         <v>52</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4850,7 +4856,7 @@
         <v>40</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4858,7 +4864,7 @@
         <v>42</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4871,7 +4877,7 @@
         <v>121</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -4908,16 +4914,16 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>169</v>
@@ -4926,73 +4932,73 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="C6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -5007,7 +5013,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
@@ -5015,18 +5021,18 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5042,12 +5048,12 @@
         <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
@@ -5055,7 +5061,7 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>128</v>
@@ -5063,18 +5069,18 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -5111,16 +5117,16 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>1</v>
@@ -5129,25 +5135,25 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="C4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>46</v>
@@ -5156,25 +5162,25 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>1</v>
@@ -5183,19 +5189,19 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>202</v>
+        <v>167</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -5210,7 +5216,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>1</v>
@@ -5218,18 +5224,18 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5245,12 +5251,12 @@
         <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>1</v>
@@ -5261,12 +5267,12 @@
         <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>204</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>1</v>
@@ -5274,7 +5280,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>1</v>
@@ -5282,10 +5288,10 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -5330,16 +5336,16 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>168</v>
+        <v>182</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>46</v>
@@ -5348,16 +5354,16 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="C5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>46</v>
@@ -5366,7 +5372,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>56</v>
@@ -5375,25 +5381,25 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>1</v>
@@ -5402,19 +5408,19 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>206</v>
+        <v>171</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -5429,7 +5435,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -5437,18 +5443,18 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5464,12 +5470,12 @@
         <v>58</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>1</v>
@@ -5480,47 +5486,47 @@
         <v>36</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>209</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -5557,28 +5563,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5596,19 +5602,19 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -5623,28 +5629,28 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -5662,16 +5668,16 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="C15" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>1</v>
@@ -5679,10 +5685,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5690,15 +5696,15 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -5735,28 +5741,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5801,10 +5807,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -5822,10 +5828,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -5834,7 +5840,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -5843,7 +5849,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>37</v>
@@ -5854,7 +5860,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5915,28 +5921,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5981,10 +5987,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -6002,10 +6008,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -6014,7 +6020,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>1</v>
@@ -6026,7 +6032,7 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6284,107 +6290,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6392,16 +6398,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>2.05</v>
@@ -6427,16 +6433,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>2.05</v>
@@ -6462,16 +6468,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>2.05</v>
@@ -6497,16 +6503,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>2.05</v>
@@ -6532,16 +6538,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>2.05</v>
@@ -6567,16 +6573,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>2.05</v>
@@ -6602,16 +6608,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>1.25</v>
@@ -6637,16 +6643,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>1.25</v>
@@ -6698,89 +6704,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6800,7 +6806,7 @@
         <v>0.5</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>300</v>
@@ -6829,7 +6835,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>300</v>
@@ -6858,7 +6864,7 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>300</v>
@@ -6887,7 +6893,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>300</v>
@@ -6916,7 +6922,7 @@
         <v>0.5</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>300</v>
@@ -6945,7 +6951,7 @@
         <v>0.5</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>300</v>
@@ -6984,44 +6990,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7029,7 +7035,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>11</v>
@@ -7043,7 +7049,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>11</v>

</xml_diff>

<commit_message>
Deployed be499d93 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Manual/source/tab/parameters.xlsx
+++ b/Manual/source/tab/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="21"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="24"/>
   </bookViews>
   <sheets>
     <sheet name="TGZ-D-48-13_26" sheetId="1" state="visible" r:id="rId3"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1509" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1511" uniqueCount="310">
   <si>
     <t xml:space="preserve">NAPÁJENÍ</t>
   </si>
@@ -686,6 +686,9 @@
     <t xml:space="preserve">3 x 400 VAC</t>
   </si>
   <si>
+    <t xml:space="preserve">32 A</t>
+  </si>
+  <si>
     <t xml:space="preserve">560 VDC</t>
   </si>
   <si>
@@ -698,7 +701,31 @@
     <t xml:space="preserve">400 W</t>
   </si>
   <si>
-    <t xml:space="preserve">32 A</t>
+    <t xml:space="preserve">9 kW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doporučené jištění</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jistič 32 A </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC IN konektor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 4pin WEIDMÜLLER BVF 7.62HP/04/180F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 6pin WEIDMÜLLER BVF 7.62HP/06/180F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 4pin WEIDMÜLLER BCZ 3.81/04/180F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brzdný odpor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 3pin WEIDMÜLLER BLZ 7.62HP/03/180F</t>
   </si>
   <si>
     <t xml:space="preserve">3 x 400 VAC/50Hz 63A</t>
@@ -3979,212 +4006,212 @@
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>165</v>
       </c>
     </row>
@@ -4207,212 +4234,212 @@
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>165</v>
       </c>
     </row>
@@ -4435,212 +4462,212 @@
   <dimension ref="A1:B31"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="45.61"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>165</v>
       </c>
     </row>
@@ -5099,7 +5126,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42.22"/>
@@ -5129,7 +5156,7 @@
         <v>182</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>211</v>
       </c>
       <c r="C3" s="3"/>
     </row>
@@ -5138,7 +5165,7 @@
         <v>183</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5147,7 +5174,7 @@
         <v>185</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -5165,7 +5192,7 @@
         <v>189</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C7" s="3"/>
     </row>
@@ -5174,7 +5201,7 @@
         <v>191</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -5183,7 +5210,7 @@
         <v>193</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>1</v>
+        <v>216</v>
       </c>
       <c r="C9" s="3"/>
     </row>
@@ -5198,10 +5225,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C11" s="3"/>
     </row>
@@ -5272,10 +5299,10 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5283,7 +5310,7 @@
         <v>206</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>1</v>
+        <v>221</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5291,7 +5318,15 @@
         <v>208</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>209</v>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -5339,7 +5374,7 @@
         <v>180</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="C3" s="3"/>
     </row>
@@ -5357,7 +5392,7 @@
         <v>183</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -5393,7 +5428,7 @@
         <v>191</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C9" s="3"/>
     </row>
@@ -5420,7 +5455,7 @@
         <v>197</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -5494,7 +5529,7 @@
         <v>205</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5515,7 +5550,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>209</v>
@@ -5523,10 +5558,10 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>220</v>
+        <v>229</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>221</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -5563,28 +5598,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5602,19 +5637,19 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="C8" s="3"/>
     </row>
@@ -5629,28 +5664,28 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="C12" s="3"/>
     </row>
@@ -5668,10 +5703,10 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="C15" s="3"/>
     </row>
@@ -5685,10 +5720,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5696,15 +5731,15 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -5741,28 +5776,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5807,10 +5842,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -5828,10 +5863,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -5849,7 +5884,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>37</v>
@@ -5860,7 +5895,7 @@
         <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5921,28 +5956,28 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>224</v>
+        <v>233</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>225</v>
+        <v>234</v>
       </c>
       <c r="C3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C4" s="3"/>
     </row>
@@ -5987,10 +6022,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="C10" s="3"/>
     </row>
@@ -6008,10 +6043,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="C13" s="3"/>
     </row>
@@ -6032,7 +6067,7 @@
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6290,107 +6325,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6398,16 +6433,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>2.05</v>
@@ -6433,16 +6468,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>2.05</v>
@@ -6468,16 +6503,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>2.05</v>
@@ -6503,16 +6538,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>2.05</v>
@@ -6538,16 +6573,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>2.05</v>
@@ -6573,16 +6608,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>2.05</v>
@@ -6608,16 +6643,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>1.25</v>
@@ -6643,16 +6678,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>24</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>1.25</v>
@@ -6704,89 +6739,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6806,7 +6841,7 @@
         <v>0.5</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>300</v>
@@ -6835,7 +6870,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>300</v>
@@ -6864,7 +6899,7 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>300</v>
@@ -6893,7 +6928,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>300</v>
@@ -6922,7 +6957,7 @@
         <v>0.5</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>300</v>
@@ -6951,7 +6986,7 @@
         <v>0.5</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>300</v>
@@ -6990,44 +7025,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7035,7 +7070,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C4" s="1" t="n">
         <v>11</v>
@@ -7049,7 +7084,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="C5" s="1" t="n">
         <v>11</v>

</xml_diff>

<commit_message>
Deployed 06b8df8b with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Manual/source/tab/parameters.xlsx
+++ b/Manual/source/tab/parameters.xlsx
@@ -713,10 +713,10 @@
     <t xml:space="preserve">AC IN konektor</t>
   </si>
   <si>
-    <t xml:space="preserve">1 x 4pin WEIDMÜLLER BVF 7.62HP/04/180F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 x 6pin WEIDMÜLLER BVF 7.62HP/06/180F</t>
+    <t xml:space="preserve">1 x 4pin WEIDMÜLLER BVZ 7.62HP/04/180F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x 6pin WEIDMÜLLER BVZ 7.62HP/06/180F</t>
   </si>
   <si>
     <t xml:space="preserve">1 x 4pin WEIDMÜLLER BCZ 3.81/04/180F</t>

</xml_diff>

<commit_message>
Deployed a9591486 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Manual/source/tab/parameters.xlsx
+++ b/Manual/source/tab/parameters.xlsx
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2253" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2253" uniqueCount="340">
   <si>
     <t xml:space="preserve">NAPÁJENÍ</t>
   </si>
@@ -853,6 +853,9 @@
   </si>
   <si>
     <t xml:space="preserve">2 x 10pin WEIDMÜLLER B2CF 3.50/10/180 SN OR BX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0–48 VDC (jištění 100 A)</t>
   </si>
   <si>
     <t xml:space="preserve">Červená/zelená dioda</t>
@@ -11734,7 +11737,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12098,7 +12101,7 @@
         <v>256</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -12537,7 +12540,7 @@
         <v>256</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C14" s="2"/>
     </row>
@@ -12601,107 +12604,107 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12709,16 +12712,16 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2.05</v>
@@ -12744,16 +12747,16 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2.05</v>
@@ -12779,16 +12782,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2.05</v>
@@ -12814,16 +12817,16 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2.05</v>
@@ -12849,16 +12852,16 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2.05</v>
@@ -12884,16 +12887,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2.05</v>
@@ -12919,16 +12922,16 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1.25</v>
@@ -12954,16 +12957,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>1.25</v>
@@ -13015,98 +13018,98 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13114,10 +13117,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>24</v>
@@ -13146,10 +13149,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>24</v>
@@ -13178,10 +13181,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>24</v>
@@ -13210,10 +13213,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>24</v>
@@ -13242,10 +13245,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>24</v>
@@ -13274,10 +13277,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>24</v>
@@ -13306,10 +13309,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>24</v>
@@ -13338,10 +13341,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>24</v>
@@ -13396,89 +13399,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13498,7 +13501,7 @@
         <v>0.5</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>300</v>
@@ -13527,7 +13530,7 @@
         <v>0.5</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>300</v>
@@ -13556,7 +13559,7 @@
         <v>0.5</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>300</v>
@@ -13585,7 +13588,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>300</v>
@@ -13614,7 +13617,7 @@
         <v>0.5</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>300</v>
@@ -13643,7 +13646,7 @@
         <v>0.5</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>300</v>
@@ -13682,44 +13685,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13727,7 +13730,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>11</v>
@@ -13741,7 +13744,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>11</v>
@@ -13792,10 +13795,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -13834,7 +13837,7 @@
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>1</v>
@@ -13842,66 +13845,66 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>